<commit_message>
Artículo: compatibilidad de libros de Excel entre equipos, con revisor en Python y lista (ES/EN, programado para el 17-dic); se limpian rutas locales de tres libros descargables
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/descargas/concurso-docente/control-documentos-aspirante.xlsx
+++ b/public/descargas/concurso-docente/control-documentos-aspirante.xlsx
@@ -4,9 +4,7 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\edwinortizNET\public\descargas\concurso-docente\"/>
-    </mc:Choice>
+    <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{40C44253-0CA4-4519-A87C-DD9ABE53FADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>

</xml_diff>